<commit_message>
policy/pm: enforce response todo closure and pivot immediate sequence to Workstream A
</commit_message>
<xml_diff>
--- a/management/docs/boilerplate-sync-candidates.xlsx
+++ b/management/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$96</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2372" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2996" uniqueCount="293">
   <si>
     <t>candidate_id</t>
   </si>
@@ -884,6 +884,18 @@
   </si>
   <si>
     <t>849</t>
+  </si>
+  <si>
+    <t>2026-02-23T22:45:11Z</t>
+  </si>
+  <si>
+    <t>2026-02-23-response-closure-policy-workstream-a-handoff</t>
+  </si>
+  <si>
+    <t>2026-02-23T22:45:02.705395659Z</t>
+  </si>
+  <si>
+    <t>432</t>
   </si>
 </sst>
 </file>
@@ -928,7 +940,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1016,7 +1028,7 @@
         <v>23</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3">
@@ -1060,7 +1072,7 @@
         <v>29</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4">
@@ -1104,7 +1116,7 @@
         <v>33</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="5">
@@ -1148,7 +1160,7 @@
         <v>29</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6">
@@ -1192,7 +1204,7 @@
         <v>40</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="7">
@@ -1236,7 +1248,7 @@
         <v>45</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="8">
@@ -1280,7 +1292,7 @@
         <v>40</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9">
@@ -1324,7 +1336,7 @@
         <v>53</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="10">
@@ -1368,7 +1380,7 @@
         <v>29</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="11">
@@ -1412,7 +1424,7 @@
         <v>33</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="12">
@@ -1456,7 +1468,7 @@
         <v>64</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="13">
@@ -1500,7 +1512,7 @@
         <v>33</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="14">
@@ -1544,7 +1556,7 @@
         <v>53</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="15">
@@ -1588,7 +1600,7 @@
         <v>21</v>
       </c>
       <c r="N15" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="16">
@@ -1632,7 +1644,7 @@
         <v>21</v>
       </c>
       <c r="N16" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="17">
@@ -1676,7 +1688,7 @@
         <v>33</v>
       </c>
       <c r="N17" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="18">
@@ -1720,7 +1732,7 @@
         <v>83</v>
       </c>
       <c r="N18" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="19">
@@ -1764,7 +1776,7 @@
         <v>87</v>
       </c>
       <c r="N19" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="20">
@@ -1808,7 +1820,7 @@
         <v>91</v>
       </c>
       <c r="N20" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="21">
@@ -1852,7 +1864,7 @@
         <v>87</v>
       </c>
       <c r="N21" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="22">
@@ -1896,15 +1908,15 @@
         <v>21</v>
       </c>
       <c r="N22" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>190</v>
+        <v>290</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>190</v>
+        <v>290</v>
       </c>
       <c r="C23" t="s" s="0">
         <v>16</v>
@@ -1913,10 +1925,10 @@
         <v>17</v>
       </c>
       <c r="E23" t="s" s="0">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="F23" t="s" s="0">
-        <v>192</v>
+        <v>97</v>
       </c>
       <c r="G23" t="s" s="0">
         <v>20</v>
@@ -1940,18 +1952,62 @@
         <v>21</v>
       </c>
       <c r="N23" t="s" s="0">
-        <v>261</v>
+        <v>289</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>190</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>190</v>
+      </c>
+      <c r="C24" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D24" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E24" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="F24" t="s" s="0">
+        <v>192</v>
+      </c>
+      <c r="G24" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="H24" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I24" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="J24" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K24" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="L24" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="M24" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="N24" t="s" s="0">
+        <v>289</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N23"/>
+  <autoFilter ref="A1:N24"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -2946,28 +3002,72 @@
     </row>
     <row r="91">
       <c r="A91" t="s" s="0">
-        <v>190</v>
+        <v>290</v>
       </c>
       <c r="B91" t="s" s="0">
         <v>100</v>
       </c>
       <c r="C91" t="s" s="0">
-        <v>193</v>
+        <v>187</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s" s="0">
+        <v>290</v>
+      </c>
+      <c r="B92" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="C92" t="s" s="0">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="s" s="0">
+        <v>290</v>
+      </c>
+      <c r="B93" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="C93" t="s" s="0">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="s" s="0">
+        <v>290</v>
+      </c>
+      <c r="B94" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="C94" t="s" s="0">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="s" s="0">
         <v>190</v>
       </c>
-      <c r="B92" t="s" s="0">
+      <c r="B95" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="C95" t="s" s="0">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="s" s="0">
+        <v>190</v>
+      </c>
+      <c r="B96" t="s" s="0">
         <v>106</v>
       </c>
-      <c r="C92" t="s" s="0">
+      <c r="C96" t="s" s="0">
         <v>194</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C92"/>
+  <autoFilter ref="A1:C96"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
pm: add active workstream A..Z presentation index with unique internal IDs
</commit_message>
<xml_diff>
--- a/management/docs/boilerplate-sync-candidates.xlsx
+++ b/management/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$100</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2996" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3646" uniqueCount="297">
   <si>
     <t>candidate_id</t>
   </si>
@@ -896,6 +896,18 @@
   </si>
   <si>
     <t>432</t>
+  </si>
+  <si>
+    <t>2026-02-23T22:57:07Z</t>
+  </si>
+  <si>
+    <t>2026-02-23-workstream-identity-presentation-aliasing</t>
+  </si>
+  <si>
+    <t>2026-02-23T22:56:57.813292472Z</t>
+  </si>
+  <si>
+    <t>403</t>
   </si>
 </sst>
 </file>
@@ -940,7 +952,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1028,7 +1040,7 @@
         <v>23</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="3">
@@ -1072,7 +1084,7 @@
         <v>29</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4">
@@ -1116,7 +1128,7 @@
         <v>33</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="5">
@@ -1160,7 +1172,7 @@
         <v>29</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="6">
@@ -1204,7 +1216,7 @@
         <v>40</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="7">
@@ -1248,7 +1260,7 @@
         <v>45</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="8">
@@ -1292,7 +1304,7 @@
         <v>40</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="9">
@@ -1336,7 +1348,7 @@
         <v>53</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="10">
@@ -1380,7 +1392,7 @@
         <v>29</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="11">
@@ -1424,7 +1436,7 @@
         <v>33</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="12">
@@ -1468,7 +1480,7 @@
         <v>64</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="13">
@@ -1512,7 +1524,7 @@
         <v>33</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="14">
@@ -1556,7 +1568,7 @@
         <v>53</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="15">
@@ -1600,7 +1612,7 @@
         <v>21</v>
       </c>
       <c r="N15" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="16">
@@ -1644,7 +1656,7 @@
         <v>21</v>
       </c>
       <c r="N16" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="17">
@@ -1688,7 +1700,7 @@
         <v>33</v>
       </c>
       <c r="N17" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="18">
@@ -1732,7 +1744,7 @@
         <v>83</v>
       </c>
       <c r="N18" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="19">
@@ -1776,7 +1788,7 @@
         <v>87</v>
       </c>
       <c r="N19" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="20">
@@ -1820,7 +1832,7 @@
         <v>91</v>
       </c>
       <c r="N20" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="21">
@@ -1864,7 +1876,7 @@
         <v>87</v>
       </c>
       <c r="N21" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="22">
@@ -1908,7 +1920,7 @@
         <v>21</v>
       </c>
       <c r="N22" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="23">
@@ -1952,7 +1964,7 @@
         <v>21</v>
       </c>
       <c r="N23" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="24">
@@ -1996,18 +2008,62 @@
         <v>21</v>
       </c>
       <c r="N24" t="s" s="0">
-        <v>289</v>
+        <v>293</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>294</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>294</v>
+      </c>
+      <c r="C25" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D25" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E25" t="s" s="0">
+        <v>295</v>
+      </c>
+      <c r="F25" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="G25" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="H25" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I25" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="J25" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K25" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="L25" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="M25" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="N25" t="s" s="0">
+        <v>293</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N24"/>
+  <autoFilter ref="A1:N25"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3066,8 +3122,52 @@
         <v>194</v>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="s" s="0">
+        <v>294</v>
+      </c>
+      <c r="B97" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="C97" t="s" s="0">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="s" s="0">
+        <v>294</v>
+      </c>
+      <c r="B98" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="C98" t="s" s="0">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="s" s="0">
+        <v>294</v>
+      </c>
+      <c r="B99" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="C99" t="s" s="0">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="s" s="0">
+        <v>294</v>
+      </c>
+      <c r="B100" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="C100" t="s" s="0">
+        <v>296</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C96"/>
+  <autoFilter ref="A1:C100"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
pm: close WS-2026-001 and publish continuation next-step deltas
</commit_message>
<xml_diff>
--- a/management/docs/boilerplate-sync-candidates.xlsx
+++ b/management/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$104</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3646" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4322" uniqueCount="301">
   <si>
     <t>candidate_id</t>
   </si>
@@ -908,6 +908,18 @@
   </si>
   <si>
     <t>403</t>
+  </si>
+  <si>
+    <t>2026-02-23T23:21:03Z</t>
+  </si>
+  <si>
+    <t>2026-02-23-ws2026-001-closeout-next-step-deltas</t>
+  </si>
+  <si>
+    <t>2026-02-23T23:15:31.497548408Z</t>
+  </si>
+  <si>
+    <t>414</t>
   </si>
 </sst>
 </file>
@@ -952,7 +964,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1040,7 +1052,7 @@
         <v>23</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="3">
@@ -1084,7 +1096,7 @@
         <v>29</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4">
@@ -1128,7 +1140,7 @@
         <v>33</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="5">
@@ -1172,7 +1184,7 @@
         <v>29</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="6">
@@ -1216,7 +1228,7 @@
         <v>40</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="7">
@@ -1260,7 +1272,7 @@
         <v>45</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="8">
@@ -1304,7 +1316,7 @@
         <v>40</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="9">
@@ -1348,7 +1360,7 @@
         <v>53</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="10">
@@ -1392,7 +1404,7 @@
         <v>29</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="11">
@@ -1436,7 +1448,7 @@
         <v>33</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="12">
@@ -1480,7 +1492,7 @@
         <v>64</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13">
@@ -1524,7 +1536,7 @@
         <v>33</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="14">
@@ -1568,7 +1580,7 @@
         <v>53</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="15">
@@ -1612,7 +1624,7 @@
         <v>21</v>
       </c>
       <c r="N15" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="16">
@@ -1656,7 +1668,7 @@
         <v>21</v>
       </c>
       <c r="N16" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="17">
@@ -1700,7 +1712,7 @@
         <v>33</v>
       </c>
       <c r="N17" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="18">
@@ -1744,7 +1756,7 @@
         <v>83</v>
       </c>
       <c r="N18" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="19">
@@ -1788,7 +1800,7 @@
         <v>87</v>
       </c>
       <c r="N19" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="20">
@@ -1832,7 +1844,7 @@
         <v>91</v>
       </c>
       <c r="N20" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="21">
@@ -1876,7 +1888,7 @@
         <v>87</v>
       </c>
       <c r="N21" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="22">
@@ -1920,7 +1932,7 @@
         <v>21</v>
       </c>
       <c r="N22" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="23">
@@ -1964,7 +1976,7 @@
         <v>21</v>
       </c>
       <c r="N23" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="24">
@@ -2008,7 +2020,7 @@
         <v>21</v>
       </c>
       <c r="N24" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
       </c>
     </row>
     <row r="25">
@@ -2052,18 +2064,62 @@
         <v>21</v>
       </c>
       <c r="N25" t="s" s="0">
-        <v>293</v>
+        <v>297</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
+        <v>298</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>298</v>
+      </c>
+      <c r="C26" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D26" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E26" t="s" s="0">
+        <v>299</v>
+      </c>
+      <c r="F26" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="G26" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="H26" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I26" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="J26" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K26" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="L26" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="M26" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="N26" t="s" s="0">
+        <v>297</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N25"/>
+  <autoFilter ref="A1:N26"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3166,8 +3222,52 @@
         <v>296</v>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="s" s="0">
+        <v>298</v>
+      </c>
+      <c r="B101" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="C101" t="s" s="0">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="s" s="0">
+        <v>298</v>
+      </c>
+      <c r="B102" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="C102" t="s" s="0">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="s" s="0">
+        <v>298</v>
+      </c>
+      <c r="B103" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="C103" t="s" s="0">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="s" s="0">
+        <v>298</v>
+      </c>
+      <c r="B104" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="C104" t="s" s="0">
+        <v>300</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C100"/>
+  <autoFilter ref="A1:C104"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
pm: enforce realm-ringfenced artifact publication
</commit_message>
<xml_diff>
--- a/management/docs/boilerplate-sync-candidates.xlsx
+++ b/management/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$108</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4322" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5024" uniqueCount="309">
   <si>
     <t>candidate_id</t>
   </si>
@@ -920,6 +920,30 @@
   </si>
   <si>
     <t>414</t>
+  </si>
+  <si>
+    <t>2026-02-24T16:41:52Z</t>
+  </si>
+  <si>
+    <t>2026-02-24-realm-artifact-ringfencing</t>
+  </si>
+  <si>
+    <t>2026-02-24T16:41:40.168932526Z</t>
+  </si>
+  <si>
+    <t>Apply realm artifact ringfencing so CI/report artifacts are indexed per realm under parent management paths rather than copied into application preview output.</t>
+  </si>
+  <si>
+    <t>273</t>
+  </si>
+  <si>
+    <t>250</t>
+  </si>
+  <si>
+    <t>253</t>
+  </si>
+  <si>
+    <t>392</t>
   </si>
 </sst>
 </file>
@@ -964,7 +988,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1052,7 +1076,7 @@
         <v>23</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="3">
@@ -1096,7 +1120,7 @@
         <v>29</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4">
@@ -1140,7 +1164,7 @@
         <v>33</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="5">
@@ -1184,7 +1208,7 @@
         <v>29</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="6">
@@ -1228,7 +1252,7 @@
         <v>40</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="7">
@@ -1272,7 +1296,7 @@
         <v>45</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="8">
@@ -1316,7 +1340,7 @@
         <v>40</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="9">
@@ -1360,7 +1384,7 @@
         <v>53</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="10">
@@ -1404,7 +1428,7 @@
         <v>29</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="11">
@@ -1448,7 +1472,7 @@
         <v>33</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="12">
@@ -1492,7 +1516,7 @@
         <v>64</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="13">
@@ -1536,7 +1560,7 @@
         <v>33</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="14">
@@ -1580,7 +1604,7 @@
         <v>53</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="15">
@@ -1624,7 +1648,7 @@
         <v>21</v>
       </c>
       <c r="N15" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="16">
@@ -1668,7 +1692,7 @@
         <v>21</v>
       </c>
       <c r="N16" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="17">
@@ -1712,7 +1736,7 @@
         <v>33</v>
       </c>
       <c r="N17" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="18">
@@ -1756,7 +1780,7 @@
         <v>83</v>
       </c>
       <c r="N18" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="19">
@@ -1800,7 +1824,7 @@
         <v>87</v>
       </c>
       <c r="N19" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="20">
@@ -1844,7 +1868,7 @@
         <v>91</v>
       </c>
       <c r="N20" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="21">
@@ -1888,7 +1912,7 @@
         <v>87</v>
       </c>
       <c r="N21" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="22">
@@ -1932,7 +1956,7 @@
         <v>21</v>
       </c>
       <c r="N22" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="23">
@@ -1976,7 +2000,7 @@
         <v>21</v>
       </c>
       <c r="N23" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="24">
@@ -2020,7 +2044,7 @@
         <v>21</v>
       </c>
       <c r="N24" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="25">
@@ -2064,7 +2088,7 @@
         <v>21</v>
       </c>
       <c r="N25" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="26">
@@ -2108,18 +2132,62 @@
         <v>21</v>
       </c>
       <c r="N26" t="s" s="0">
-        <v>297</v>
+        <v>301</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C27" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D27" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E27" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="F27" t="s" s="0">
+        <v>304</v>
+      </c>
+      <c r="G27" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="H27" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I27" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="J27" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K27" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="L27" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="M27" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="N27" t="s" s="0">
+        <v>301</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N26"/>
+  <autoFilter ref="A1:N27"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C108"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3266,8 +3334,52 @@
         <v>300</v>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="B105" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="C105" t="s" s="0">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="B106" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="C106" t="s" s="0">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="B107" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="C107" t="s" s="0">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="B108" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="C108" t="s" s="0">
+        <v>308</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C104"/>
+  <autoFilter ref="A1:C108"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
build: ingest all sampleData AFP files into sampleOutput during build
</commit_message>
<xml_diff>
--- a/management/docs/boilerplate-sync-candidates.xlsx
+++ b/management/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$112</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5024" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5752" uniqueCount="316">
   <si>
     <t>candidate_id</t>
   </si>
@@ -944,6 +944,27 @@
   </si>
   <si>
     <t>392</t>
+  </si>
+  <si>
+    <t>2026-02-24T16:51:53Z</t>
+  </si>
+  <si>
+    <t>2026-02-24-sampledata-build-ingestion</t>
+  </si>
+  <si>
+    <t>2026-02-24T16:51:44.685590008Z</t>
+  </si>
+  <si>
+    <t>Propagate build-task behavior that ingests all AFP files under `product/afp-converter/sampleData` and generates corresponding sample outputs during build.</t>
+  </si>
+  <si>
+    <t>268</t>
+  </si>
+  <si>
+    <t>262</t>
+  </si>
+  <si>
+    <t>145</t>
   </si>
 </sst>
 </file>
@@ -988,7 +1009,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1076,7 +1097,7 @@
         <v>23</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="3">
@@ -1120,7 +1141,7 @@
         <v>29</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4">
@@ -1164,7 +1185,7 @@
         <v>33</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="5">
@@ -1208,7 +1229,7 @@
         <v>29</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="6">
@@ -1252,7 +1273,7 @@
         <v>40</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="7">
@@ -1296,7 +1317,7 @@
         <v>45</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="8">
@@ -1340,7 +1361,7 @@
         <v>40</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="9">
@@ -1384,7 +1405,7 @@
         <v>53</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="10">
@@ -1428,7 +1449,7 @@
         <v>29</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="11">
@@ -1472,7 +1493,7 @@
         <v>33</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="12">
@@ -1516,7 +1537,7 @@
         <v>64</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="13">
@@ -1560,7 +1581,7 @@
         <v>33</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="14">
@@ -1604,7 +1625,7 @@
         <v>53</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="15">
@@ -1648,7 +1669,7 @@
         <v>21</v>
       </c>
       <c r="N15" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="16">
@@ -1692,7 +1713,7 @@
         <v>21</v>
       </c>
       <c r="N16" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="17">
@@ -1736,7 +1757,7 @@
         <v>33</v>
       </c>
       <c r="N17" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="18">
@@ -1780,7 +1801,7 @@
         <v>83</v>
       </c>
       <c r="N18" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="19">
@@ -1824,7 +1845,7 @@
         <v>87</v>
       </c>
       <c r="N19" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="20">
@@ -1868,7 +1889,7 @@
         <v>91</v>
       </c>
       <c r="N20" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="21">
@@ -1912,7 +1933,7 @@
         <v>87</v>
       </c>
       <c r="N21" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="22">
@@ -1956,7 +1977,7 @@
         <v>21</v>
       </c>
       <c r="N22" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="23">
@@ -2000,7 +2021,7 @@
         <v>21</v>
       </c>
       <c r="N23" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="24">
@@ -2044,7 +2065,7 @@
         <v>21</v>
       </c>
       <c r="N24" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="25">
@@ -2088,7 +2109,7 @@
         <v>21</v>
       </c>
       <c r="N25" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="26">
@@ -2132,7 +2153,7 @@
         <v>21</v>
       </c>
       <c r="N26" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="27">
@@ -2176,18 +2197,62 @@
         <v>21</v>
       </c>
       <c r="N27" t="s" s="0">
-        <v>301</v>
+        <v>309</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="C28" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D28" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E28" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="F28" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="G28" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="H28" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I28" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="J28" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K28" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="L28" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="M28" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="N28" t="s" s="0">
+        <v>309</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N27"/>
+  <autoFilter ref="A1:N28"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3378,8 +3443,52 @@
         <v>308</v>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="B109" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="C109" t="s" s="0">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="B110" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="C110" t="s" s="0">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="B111" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="C111" t="s" s="0">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="B112" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="C112" t="s" s="0">
+        <v>159</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C108"/>
+  <autoFilter ref="A1:C112"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: protect sampleOutput baselines and reroute generated sample outputs
</commit_message>
<xml_diff>
--- a/management/docs/boilerplate-sync-candidates.xlsx
+++ b/management/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$116</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5752" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6506" uniqueCount="322">
   <si>
     <t>candidate_id</t>
   </si>
@@ -965,6 +965,24 @@
   </si>
   <si>
     <t>145</t>
+  </si>
+  <si>
+    <t>2026-02-24T17:01:19Z</t>
+  </si>
+  <si>
+    <t>2026-02-24-sample-baseline-protection-correction</t>
+  </si>
+  <si>
+    <t>2026-02-24T17:00:44.932146668Z</t>
+  </si>
+  <si>
+    <t>Correct sample artifact handling so baseline comparison files in `sampleOutput` are protected, while generated multi-sample outputs are emitted under preview paths.</t>
+  </si>
+  <si>
+    <t>278</t>
+  </si>
+  <si>
+    <t>433</t>
   </si>
 </sst>
 </file>
@@ -1009,7 +1027,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1097,7 +1115,7 @@
         <v>23</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="3">
@@ -1141,7 +1159,7 @@
         <v>29</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="4">
@@ -1185,7 +1203,7 @@
         <v>33</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5">
@@ -1229,7 +1247,7 @@
         <v>29</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="6">
@@ -1273,7 +1291,7 @@
         <v>40</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="7">
@@ -1317,7 +1335,7 @@
         <v>45</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="8">
@@ -1361,7 +1379,7 @@
         <v>40</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="9">
@@ -1405,7 +1423,7 @@
         <v>53</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="10">
@@ -1449,7 +1467,7 @@
         <v>29</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="11">
@@ -1493,7 +1511,7 @@
         <v>33</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="12">
@@ -1537,7 +1555,7 @@
         <v>64</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="13">
@@ -1581,7 +1599,7 @@
         <v>33</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="14">
@@ -1625,7 +1643,7 @@
         <v>53</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="15">
@@ -1669,7 +1687,7 @@
         <v>21</v>
       </c>
       <c r="N15" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="16">
@@ -1713,7 +1731,7 @@
         <v>21</v>
       </c>
       <c r="N16" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="17">
@@ -1757,7 +1775,7 @@
         <v>33</v>
       </c>
       <c r="N17" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="18">
@@ -1801,7 +1819,7 @@
         <v>83</v>
       </c>
       <c r="N18" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="19">
@@ -1845,7 +1863,7 @@
         <v>87</v>
       </c>
       <c r="N19" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="20">
@@ -1889,7 +1907,7 @@
         <v>91</v>
       </c>
       <c r="N20" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="21">
@@ -1933,7 +1951,7 @@
         <v>87</v>
       </c>
       <c r="N21" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="22">
@@ -1977,7 +1995,7 @@
         <v>21</v>
       </c>
       <c r="N22" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="23">
@@ -2021,7 +2039,7 @@
         <v>21</v>
       </c>
       <c r="N23" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="24">
@@ -2065,7 +2083,7 @@
         <v>21</v>
       </c>
       <c r="N24" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="25">
@@ -2109,7 +2127,7 @@
         <v>21</v>
       </c>
       <c r="N25" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="26">
@@ -2153,7 +2171,7 @@
         <v>21</v>
       </c>
       <c r="N26" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="27">
@@ -2197,15 +2215,15 @@
         <v>21</v>
       </c>
       <c r="N27" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="C28" t="s" s="0">
         <v>16</v>
@@ -2214,10 +2232,10 @@
         <v>17</v>
       </c>
       <c r="E28" t="s" s="0">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="F28" t="s" s="0">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="G28" t="s" s="0">
         <v>20</v>
@@ -2241,18 +2259,62 @@
         <v>21</v>
       </c>
       <c r="N28" t="s" s="0">
-        <v>309</v>
+        <v>316</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="C29" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D29" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E29" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="F29" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="G29" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="H29" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I29" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="J29" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K29" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="L29" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="M29" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="N29" t="s" s="0">
+        <v>316</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N28"/>
+  <autoFilter ref="A1:N29"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C116"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3445,50 +3507,94 @@
     </row>
     <row r="109">
       <c r="A109" t="s" s="0">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B109" t="s" s="0">
         <v>100</v>
       </c>
       <c r="C109" t="s" s="0">
-        <v>313</v>
+        <v>320</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="s" s="0">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B110" t="s" s="0">
         <v>102</v>
       </c>
       <c r="C110" t="s" s="0">
-        <v>314</v>
+        <v>145</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s" s="0">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B111" t="s" s="0">
         <v>104</v>
       </c>
       <c r="C111" t="s" s="0">
-        <v>315</v>
+        <v>176</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s" s="0">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B112" t="s" s="0">
         <v>106</v>
       </c>
       <c r="C112" t="s" s="0">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="B113" t="s" s="0">
+        <v>100</v>
+      </c>
+      <c r="C113" t="s" s="0">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="B114" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="C114" t="s" s="0">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="B115" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="C115" t="s" s="0">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="B116" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="C116" t="s" s="0">
         <v>159</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C112"/>
+  <autoFilter ref="A1:C116"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>